<commit_message>
6 new achievements Part 1 added
</commit_message>
<xml_diff>
--- a/Achievement Tracker.xlsx
+++ b/Achievement Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr showInkAnnotation="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jordan Leich\Documents\GitHub\Improved-Unlockables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cprin\OneDrive\Documents\GitHub\Improved-Unlockables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FEC292-F495-4447-AC60-8ADAEB240FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41DF0FD4-EF5C-4CD2-8D57-E32FF25D9ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracker!$A$1:$B$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracker!$A$1:$B$60</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>Achievement Name</t>
   </si>
@@ -206,10 +206,25 @@
     <t>Percentage Complete</t>
   </si>
   <si>
-    <t>Super Computer (Custom Achievement)</t>
-  </si>
-  <si>
     <t>The Sound of Insanity (Custom Achievement)</t>
+  </si>
+  <si>
+    <t>Train Wreck (Custom Achievement)</t>
+  </si>
+  <si>
+    <t>Database Destruction (Custom Achievement)</t>
+  </si>
+  <si>
+    <t>The Eye of the Shadow Queen (Custom Achievement)</t>
+  </si>
+  <si>
+    <t>Miscommunication (Custom Achievement)</t>
+  </si>
+  <si>
+    <t>Weapons of War (Custom Achievement)</t>
+  </si>
+  <si>
+    <t>Protection from Doom (Custom Achievement)</t>
   </si>
 </sst>
 </file>
@@ -305,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -343,6 +358,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -485,8 +503,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73806510-1F6C-4AC8-8B2C-27038AAB5244}" name="Table1" displayName="Table1" ref="A1:B56" totalsRowCount="1" headerRowDxfId="7" dataDxfId="6" totalsRowDxfId="4" tableBorderDxfId="5">
-  <autoFilter ref="A1:B55" xr:uid="{FF66C5D9-ED34-8F49-9B1C-C38D8DEA47EB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73806510-1F6C-4AC8-8B2C-27038AAB5244}" name="Table1" displayName="Table1" ref="A1:B61" totalsRowCount="1" headerRowDxfId="7" dataDxfId="6" totalsRowDxfId="4" tableBorderDxfId="5">
+  <autoFilter ref="A1:B60" xr:uid="{FF66C5D9-ED34-8F49-9B1C-C38D8DEA47EB}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{C321B8E8-0265-46CB-984A-86660BB68D40}" name="Achievement Name" totalsRowLabel="Total" dataDxfId="3" totalsRowDxfId="1"/>
     <tableColumn id="2" xr3:uid="{4A463D9A-9910-4C6B-83BA-16664CDACDE1}" name="Unlocked" totalsRowFunction="count" dataDxfId="2" totalsRowDxfId="0"/>
@@ -795,10 +813,10 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="49.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
@@ -823,7 +841,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="11">
-        <f>COUNTIF(B2:B55, TRUE) / COUNTA(A2:A55) * 100</f>
+        <f>COUNTIF(B2:B60, TRUE) / COUNTA(A2:A60) * 100</f>
         <v>0</v>
       </c>
     </row>
@@ -1229,7 +1247,7 @@
     </row>
     <row r="53" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B53" s="9" t="b">
         <v>0</v>
@@ -1237,7 +1255,7 @@
     </row>
     <row r="54" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B54" s="9" t="b">
         <v>0</v>
@@ -1245,19 +1263,59 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B57" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B58" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B59" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B55" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="7" t="s">
+      <c r="B60" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B56" s="1">
+      <c r="B61" s="1">
         <f>SUBTOTAL(103,Table1[Unlocked])</f>
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1 new achievement added
</commit_message>
<xml_diff>
--- a/Achievement Tracker.xlsx
+++ b/Achievement Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cprin\OneDrive\Documents\GitHub\Improved-Unlockables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{057B424B-ED6A-4A9C-A891-8AAC9F0FD59D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90B3A55-56D9-460E-902A-C68D908A11DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracker!$A$1:$B$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracker!$A$1:$B$61</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>Achievement Name</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>Protection from Doom (Custom Achievement)</t>
+  </si>
+  <si>
+    <t>Civil War (Custom Achievement)</t>
   </si>
 </sst>
 </file>
@@ -271,7 +274,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -293,6 +296,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -363,15 +372,35 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -390,15 +419,12 @@
         <scheme val="minor"/>
       </font>
       <fill>
-        <patternFill patternType="none">
-          <fgColor rgb="FFD9E1F2"/>
-          <bgColor auto="1"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -442,9 +468,6 @@
           <color rgb="FF8EA9DB"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -507,11 +530,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73806510-1F6C-4AC8-8B2C-27038AAB5244}" name="Table1" displayName="Table1" ref="A1:B61" totalsRowCount="1" headerRowDxfId="7" dataDxfId="6" totalsRowDxfId="4" tableBorderDxfId="5">
-  <autoFilter ref="A1:B60" xr:uid="{FF66C5D9-ED34-8F49-9B1C-C38D8DEA47EB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73806510-1F6C-4AC8-8B2C-27038AAB5244}" name="Table1" displayName="Table1" ref="A1:B62" totalsRowCount="1" headerRowDxfId="7" dataDxfId="6" totalsRowDxfId="0" tableBorderDxfId="5">
+  <autoFilter ref="A1:B61" xr:uid="{FF66C5D9-ED34-8F49-9B1C-C38D8DEA47EB}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C321B8E8-0265-46CB-984A-86660BB68D40}" name="Achievement Name" totalsRowLabel="Total" dataDxfId="3" totalsRowDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{4A463D9A-9910-4C6B-83BA-16664CDACDE1}" name="Unlocked" totalsRowFunction="count" dataDxfId="2" totalsRowDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{C321B8E8-0265-46CB-984A-86660BB68D40}" name="Achievement Name" totalsRowLabel="Total" dataDxfId="4" totalsRowDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{4A463D9A-9910-4C6B-83BA-16664CDACDE1}" name="Unlocked" totalsRowFunction="count" dataDxfId="3" totalsRowDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -817,7 +840,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -845,7 +868,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="10">
-        <f>COUNTIF(B2:B60, TRUE) / COUNTA(A2:A60) * 100</f>
+        <f>COUNTIF(B2:B61, TRUE) / COUNTA(A2:A61) * 100</f>
         <v>0</v>
       </c>
     </row>
@@ -1089,7 +1112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>32</v>
       </c>
@@ -1097,7 +1120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>33</v>
       </c>
@@ -1105,7 +1128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>34</v>
       </c>
@@ -1113,7 +1136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>35</v>
       </c>
@@ -1121,7 +1144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>36</v>
       </c>
@@ -1129,7 +1152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>37</v>
       </c>
@@ -1137,7 +1160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>38</v>
       </c>
@@ -1145,7 +1168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>39</v>
       </c>
@@ -1153,7 +1176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>40</v>
       </c>
@@ -1161,7 +1184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>41</v>
       </c>
@@ -1169,7 +1192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>42</v>
       </c>
@@ -1177,7 +1200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>43</v>
       </c>
@@ -1185,16 +1208,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="12" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
         <v>44</v>
       </c>
       <c r="B45" s="8" t="b">
         <v>0</v>
       </c>
-      <c r="C45" s="13"/>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>45</v>
       </c>
@@ -1202,15 +1224,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="12" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
         <v>46</v>
       </c>
       <c r="B47" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>47</v>
       </c>
@@ -1218,15 +1240,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="12" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
         <v>48</v>
       </c>
       <c r="B49" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>49</v>
       </c>
@@ -1234,15 +1256,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="12" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
         <v>50</v>
       </c>
       <c r="B51" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>51</v>
       </c>
@@ -1250,16 +1272,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="12" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="4" t="s">
         <v>58</v>
       </c>
       <c r="B53" s="8" t="b">
         <v>0</v>
       </c>
-      <c r="D53" s="13"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>56</v>
       </c>
@@ -1267,15 +1288,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="12" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
         <v>57</v>
       </c>
       <c r="B55" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
         <v>59</v>
       </c>
@@ -1283,15 +1304,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="12" t="s">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
         <v>60</v>
       </c>
       <c r="B57" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>61</v>
       </c>
@@ -1299,29 +1320,37 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="12" t="s">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
         <v>62</v>
       </c>
       <c r="B59" s="8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="3" t="s">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B60" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B60" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="14" t="s">
+      <c r="B61" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B61" s="1">
+      <c r="B62" s="14">
         <f>SUBTOTAL(103,Table1[Unlocked])</f>
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>